<commit_message>
Add 4 new POs to Kashif buying sheet (17257, 17308, 1194, 406)
Added Janitorial/Cleaning (28 items), Grocery/Entertainment (8 items),
Production Consumables (1 item), and Mechanical Items (1 item).
Sheet now covers 10 POs total.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JrgSPE8qZmAUatRmCqrXMY
</commit_message>
<xml_diff>
--- a/Kashif_Buying_Sheet.xlsx
+++ b/Kashif_Buying_Sheet.xlsx
@@ -61,7 +61,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -102,6 +102,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8CECC"/>
         <bgColor rgb="00F8CECC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAEEF3"/>
+        <bgColor rgb="00DAEEF3"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -202,6 +226,54 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -588,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -612,7 +684,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Date: 02-Jul-2026 &amp; 29-Jun-2026 | Deliver To: Main Store, Plot #8 Sector 27, Karachi</t>
+          <t>Dates: 29-Jun to 06-Jul-2026 | 10 POs | Deliver To: Main Store, Plot #8 Sector 27, Karachi</t>
         </is>
       </c>
     </row>
@@ -1943,201 +2015,1702 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="20" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🧹  JANITORIAL / CLEANING ITEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="21" t="n">
+        <v>36</v>
+      </c>
+      <c r="B44" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>Air Freshner Room Spray 300ml Topic Brand</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E44" s="21" t="n">
+        <v>96</v>
+      </c>
+      <c r="F44" s="23" t="n">
+        <v>260</v>
+      </c>
+      <c r="G44" s="23" t="n">
+        <v>24960</v>
+      </c>
+      <c r="H44" s="23" t="n">
+        <v>1248</v>
+      </c>
+      <c r="I44" s="23" t="n">
+        <v>26208</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="21" t="n">
+        <v>37</v>
+      </c>
+      <c r="B45" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>Bleach 30KG Local</t>
+        </is>
+      </c>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="E45" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="F45" s="23" t="n">
+        <v>970</v>
+      </c>
+      <c r="G45" s="23" t="n">
+        <v>13580</v>
+      </c>
+      <c r="H45" s="23" t="n">
+        <v>679</v>
+      </c>
+      <c r="I45" s="23" t="n">
+        <v>14259</v>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="21" t="n">
+        <v>38</v>
+      </c>
+      <c r="B46" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>Broom Hard</t>
+        </is>
+      </c>
+      <c r="D46" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E46" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="F46" s="23" t="n">
+        <v>235</v>
+      </c>
+      <c r="G46" s="23" t="n">
+        <v>47000</v>
+      </c>
+      <c r="H46" s="23" t="n">
+        <v>2350</v>
+      </c>
+      <c r="I46" s="23" t="n">
+        <v>49350</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="21" t="n">
+        <v>39</v>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>Broom Soft PP</t>
+        </is>
+      </c>
+      <c r="D47" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E47" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="F47" s="23" t="n">
+        <v>200</v>
+      </c>
+      <c r="G47" s="23" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H47" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" s="23" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>China Brush</t>
+        </is>
+      </c>
+      <c r="D48" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>60</v>
+      </c>
+      <c r="F48" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="G48" s="23" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H48" s="23" t="n">
+        <v>900</v>
+      </c>
+      <c r="I48" s="23" t="n">
+        <v>18900</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="21" t="n">
+        <v>41</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>Dustbin Bag 18x24 Black</t>
+        </is>
+      </c>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E49" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="F49" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="G49" s="23" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H49" s="23" t="n">
+        <v>750</v>
+      </c>
+      <c r="I49" s="23" t="n">
+        <v>15750</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="21" t="n">
+        <v>42</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>Dustbin Bag 30x50 Black</t>
+        </is>
+      </c>
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E50" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="F50" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="G50" s="23" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H50" s="23" t="n">
+        <v>750</v>
+      </c>
+      <c r="I50" s="23" t="n">
+        <v>15750</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="21" t="n">
+        <v>43</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>Duster Fabric</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E51" s="21" t="n">
+        <v>96</v>
+      </c>
+      <c r="F51" s="23" t="n">
+        <v>37</v>
+      </c>
+      <c r="G51" s="23" t="n">
+        <v>3552</v>
+      </c>
+      <c r="H51" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="23" t="n">
+        <v>3552</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="21" t="n">
+        <v>44</v>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>Glass Cleaner Glint 500ml</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="inlineStr">
+        <is>
+          <t>BTL</t>
+        </is>
+      </c>
+      <c r="E52" s="21" t="n">
+        <v>96</v>
+      </c>
+      <c r="F52" s="23" t="n">
+        <v>250</v>
+      </c>
+      <c r="G52" s="23" t="n">
+        <v>24000</v>
+      </c>
+      <c r="H52" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="23" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="21" t="n">
+        <v>45</v>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Hand Brush</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E53" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="F53" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="G53" s="23" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H53" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I53" s="23" t="n">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="21" t="n">
+        <v>46</v>
+      </c>
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="inlineStr">
+        <is>
+          <t>Hand Wash Lose Local</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E54" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="F54" s="23" t="n">
+        <v>270</v>
+      </c>
+      <c r="G54" s="23" t="n">
+        <v>54000</v>
+      </c>
+      <c r="H54" s="23" t="n">
+        <v>2700</v>
+      </c>
+      <c r="I54" s="23" t="n">
+        <v>56700</v>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="21" t="n">
+        <v>47</v>
+      </c>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>Handwash Lifeboy 140ml</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>BTL</t>
+        </is>
+      </c>
+      <c r="E55" s="21" t="n">
+        <v>48</v>
+      </c>
+      <c r="F55" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="G55" s="23" t="n">
+        <v>14400</v>
+      </c>
+      <c r="H55" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I55" s="23" t="n">
+        <v>14400</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="21" t="n">
+        <v>48</v>
+      </c>
+      <c r="B56" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>Harpic 500ml</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>BTL</t>
+        </is>
+      </c>
+      <c r="E56" s="21" t="n">
+        <v>96</v>
+      </c>
+      <c r="F56" s="23" t="n">
+        <v>380</v>
+      </c>
+      <c r="G56" s="23" t="n">
+        <v>36480</v>
+      </c>
+      <c r="H56" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I56" s="23" t="n">
+        <v>36480</v>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="21" t="n">
+        <v>49</v>
+      </c>
+      <c r="B57" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>Lux Soap 70 Grams</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E57" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F57" s="23" t="n">
+        <v>150</v>
+      </c>
+      <c r="G57" s="23" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H57" s="23" t="n">
+        <v>750</v>
+      </c>
+      <c r="I57" s="23" t="n">
+        <v>15750</v>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="B58" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>Mop Big 18x18 Wooden</t>
+        </is>
+      </c>
+      <c r="D58" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E58" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F58" s="23" t="n">
+        <v>394</v>
+      </c>
+      <c r="G58" s="23" t="n">
+        <v>39400</v>
+      </c>
+      <c r="H58" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I58" s="23" t="n">
+        <v>39400</v>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="21" t="n">
+        <v>51</v>
+      </c>
+      <c r="B59" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C59" s="22" t="inlineStr">
+        <is>
+          <t>Mop Refill (600 Gram)</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E59" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="F59" s="23" t="n">
+        <v>347</v>
+      </c>
+      <c r="G59" s="23" t="n">
+        <v>69400</v>
+      </c>
+      <c r="H59" s="23" t="n">
+        <v>3470</v>
+      </c>
+      <c r="I59" s="23" t="n">
+        <v>72870</v>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="21" t="n">
+        <v>52</v>
+      </c>
+      <c r="B60" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C60" s="22" t="inlineStr">
+        <is>
+          <t>Mop Stick</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E60" s="21" t="n">
+        <v>60</v>
+      </c>
+      <c r="F60" s="23" t="n">
+        <v>473</v>
+      </c>
+      <c r="G60" s="23" t="n">
+        <v>28380</v>
+      </c>
+      <c r="H60" s="23" t="n">
+        <v>1419</v>
+      </c>
+      <c r="I60" s="23" t="n">
+        <v>29799</v>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="21" t="n">
+        <v>53</v>
+      </c>
+      <c r="B61" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C61" s="22" t="inlineStr">
+        <is>
+          <t>Mortein Spray</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E61" s="21" t="n">
+        <v>48</v>
+      </c>
+      <c r="F61" s="23" t="n">
+        <v>590</v>
+      </c>
+      <c r="G61" s="23" t="n">
+        <v>28320</v>
+      </c>
+      <c r="H61" s="23" t="n">
+        <v>1416</v>
+      </c>
+      <c r="I61" s="23" t="n">
+        <v>29736</v>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="21" t="n">
+        <v>54</v>
+      </c>
+      <c r="B62" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>Phenyl Zip Local 3 Ltr</t>
+        </is>
+      </c>
+      <c r="D62" s="21" t="inlineStr">
+        <is>
+          <t>BTL</t>
+        </is>
+      </c>
+      <c r="E62" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="F62" s="23" t="n">
+        <v>420</v>
+      </c>
+      <c r="G62" s="23" t="n">
+        <v>84000</v>
+      </c>
+      <c r="H62" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="23" t="n">
+        <v>84000</v>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="B63" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C63" s="22" t="inlineStr">
+        <is>
+          <t>Roomi Box</t>
+        </is>
+      </c>
+      <c r="D63" s="21" t="inlineStr">
+        <is>
+          <t>CTN</t>
+        </is>
+      </c>
+      <c r="E63" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" s="23" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G63" s="23" t="n">
+        <v>36000</v>
+      </c>
+      <c r="H63" s="23" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I63" s="23" t="n">
+        <v>37800</v>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="21" t="n">
+        <v>56</v>
+      </c>
+      <c r="B64" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C64" s="22" t="inlineStr">
+        <is>
+          <t>Safety Match 10 PCS</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="E64" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="F64" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="G64" s="23" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H64" s="23" t="n">
+        <v>75</v>
+      </c>
+      <c r="I64" s="23" t="n">
+        <v>1575</v>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="21" t="n">
+        <v>57</v>
+      </c>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="inlineStr">
+        <is>
+          <t>Scotch Bright</t>
+        </is>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E65" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="F65" s="23" t="n">
+        <v>70</v>
+      </c>
+      <c r="G65" s="23" t="n">
+        <v>1680</v>
+      </c>
+      <c r="H65" s="23" t="n">
+        <v>84</v>
+      </c>
+      <c r="I65" s="23" t="n">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="21" t="n">
+        <v>58</v>
+      </c>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C66" s="22" t="inlineStr">
+        <is>
+          <t>Scraper Plastic Supri</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E66" s="21" t="n">
+        <v>60</v>
+      </c>
+      <c r="F66" s="23" t="n">
+        <v>105</v>
+      </c>
+      <c r="G66" s="23" t="n">
+        <v>6300</v>
+      </c>
+      <c r="H66" s="23" t="n">
+        <v>315</v>
+      </c>
+      <c r="I66" s="23" t="n">
+        <v>6615</v>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="21" t="n">
+        <v>59</v>
+      </c>
+      <c r="B67" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C67" s="22" t="inlineStr">
+        <is>
+          <t>Tile Wash Sweep Local 30KG</t>
+        </is>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="E67" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="F67" s="23" t="n">
+        <v>1180</v>
+      </c>
+      <c r="G67" s="23" t="n">
+        <v>8260</v>
+      </c>
+      <c r="H67" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="23" t="n">
+        <v>8260</v>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="21" t="n">
+        <v>60</v>
+      </c>
+      <c r="B68" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C68" s="22" t="inlineStr">
+        <is>
+          <t>Tissue Box Rose Petal Pop Up 150 Sheet</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="E68" s="21" t="n">
+        <v>150</v>
+      </c>
+      <c r="F68" s="23" t="n">
+        <v>270</v>
+      </c>
+      <c r="G68" s="23" t="n">
+        <v>40500</v>
+      </c>
+      <c r="H68" s="23" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I68" s="23" t="n">
+        <v>42525</v>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="21" t="n">
+        <v>61</v>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C69" s="22" t="inlineStr">
+        <is>
+          <t>Tissue Paper Roll</t>
+        </is>
+      </c>
+      <c r="D69" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E69" s="21" t="n">
+        <v>300</v>
+      </c>
+      <c r="F69" s="23" t="n">
+        <v>120</v>
+      </c>
+      <c r="G69" s="23" t="n">
+        <v>36000</v>
+      </c>
+      <c r="H69" s="23" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I69" s="23" t="n">
+        <v>37800</v>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="21" t="n">
+        <v>62</v>
+      </c>
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C70" s="22" t="inlineStr">
+        <is>
+          <t>VIM Toilet Bleach Powder Lose Local</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E70" s="21" t="n">
+        <v>25</v>
+      </c>
+      <c r="F70" s="23" t="n">
+        <v>180</v>
+      </c>
+      <c r="G70" s="23" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H70" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="23" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="21" t="n">
+        <v>63</v>
+      </c>
+      <c r="B71" s="21" t="inlineStr">
+        <is>
+          <t>17257</t>
+        </is>
+      </c>
+      <c r="C71" s="22" t="inlineStr">
+        <is>
+          <t>Viper Large 4ft</t>
+        </is>
+      </c>
+      <c r="D71" s="21" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E71" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="F71" s="23" t="n">
+        <v>579</v>
+      </c>
+      <c r="G71" s="23" t="n">
+        <v>28950</v>
+      </c>
+      <c r="H71" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="23" t="n">
+        <v>28950</v>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🛒  GROCERY / ENTERTAINMENT ITEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="25" t="n">
+        <v>64</v>
+      </c>
+      <c r="B73" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C73" s="26" t="inlineStr">
+        <is>
+          <t>Coffee (100g)</t>
+        </is>
+      </c>
+      <c r="D73" s="25" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E73" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G73" s="27" t="n">
+        <v>4800</v>
+      </c>
+      <c r="H73" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="27" t="n">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="25" t="n">
+        <v>65</v>
+      </c>
+      <c r="B74" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C74" s="26" t="inlineStr">
+        <is>
+          <t>Every Day Tea Whitener 2KG Pouch</t>
+        </is>
+      </c>
+      <c r="D74" s="25" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="E74" s="25" t="n">
+        <v>260</v>
+      </c>
+      <c r="F74" s="27" t="n">
+        <v>4185</v>
+      </c>
+      <c r="G74" s="27" t="n">
+        <v>1088100</v>
+      </c>
+      <c r="H74" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="27" t="n">
+        <v>1088100</v>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="25" t="n">
+        <v>66</v>
+      </c>
+      <c r="B75" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C75" s="26" t="inlineStr">
+        <is>
+          <t>Lipton Lemon Green Tea 100 Bags</t>
+        </is>
+      </c>
+      <c r="D75" s="25" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="E75" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F75" s="27" t="n">
+        <v>1150</v>
+      </c>
+      <c r="G75" s="27" t="n">
+        <v>34500</v>
+      </c>
+      <c r="H75" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I75" s="27" t="n">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="25" t="n">
+        <v>67</v>
+      </c>
+      <c r="B76" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C76" s="26" t="inlineStr">
+        <is>
+          <t>Lipton Tea Bag 600 Bags</t>
+        </is>
+      </c>
+      <c r="D76" s="25" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="E76" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="F76" s="27" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G76" s="27" t="n">
+        <v>36300</v>
+      </c>
+      <c r="H76" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I76" s="27" t="n">
+        <v>36300</v>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="25" t="n">
+        <v>68</v>
+      </c>
+      <c r="B77" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C77" s="26" t="inlineStr">
+        <is>
+          <t>Nescafe (200gm)</t>
+        </is>
+      </c>
+      <c r="D77" s="25" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E77" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="F77" s="27" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G77" s="27" t="n">
+        <v>50400</v>
+      </c>
+      <c r="H77" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I77" s="27" t="n">
+        <v>50400</v>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="25" t="n">
+        <v>69</v>
+      </c>
+      <c r="B78" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C78" s="26" t="inlineStr">
+        <is>
+          <t>Nestle Water 500ml</t>
+        </is>
+      </c>
+      <c r="D78" s="25" t="inlineStr">
+        <is>
+          <t>CRT</t>
+        </is>
+      </c>
+      <c r="E78" s="25" t="n">
+        <v>23</v>
+      </c>
+      <c r="F78" s="27" t="n">
+        <v>680</v>
+      </c>
+      <c r="G78" s="27" t="n">
+        <v>15640</v>
+      </c>
+      <c r="H78" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I78" s="27" t="n">
+        <v>15640</v>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="B79" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C79" s="26" t="inlineStr">
+        <is>
+          <t>Sugar 2 KGS Pack</t>
+        </is>
+      </c>
+      <c r="D79" s="25" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="E79" s="25" t="n">
+        <v>350</v>
+      </c>
+      <c r="F79" s="27" t="n">
+        <v>305</v>
+      </c>
+      <c r="G79" s="27" t="n">
+        <v>106750</v>
+      </c>
+      <c r="H79" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I79" s="27" t="n">
+        <v>106750</v>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="25" t="n">
+        <v>71</v>
+      </c>
+      <c r="B80" s="25" t="inlineStr">
+        <is>
+          <t>17308</t>
+        </is>
+      </c>
+      <c r="C80" s="26" t="inlineStr">
+        <is>
+          <t>Tapal Family Mixture (900gm)</t>
+        </is>
+      </c>
+      <c r="D80" s="25" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="E80" s="25" t="n">
+        <v>176</v>
+      </c>
+      <c r="F80" s="27" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G80" s="27" t="n">
+        <v>325600</v>
+      </c>
+      <c r="H80" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" s="27" t="n">
+        <v>325600</v>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🏭  PRODUCTION CONSUMABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="29" t="n">
+        <v>72</v>
+      </c>
+      <c r="B82" s="29" t="inlineStr">
+        <is>
+          <t>1194</t>
+        </is>
+      </c>
+      <c r="C82" s="30" t="inlineStr">
+        <is>
+          <t>Molty Foam Sheet (3'x6'x2") 980</t>
+        </is>
+      </c>
+      <c r="D82" s="29" t="inlineStr">
+        <is>
+          <t>SHT</t>
+        </is>
+      </c>
+      <c r="E82" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="F82" s="31" t="n">
+        <v>3579</v>
+      </c>
+      <c r="G82" s="31" t="n">
+        <v>21474</v>
+      </c>
+      <c r="H82" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="31" t="n">
+        <v>21474</v>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⚙️  MECHANICAL ITEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="33" t="n">
+        <v>73</v>
+      </c>
+      <c r="B84" s="33" t="inlineStr">
+        <is>
+          <t>406</t>
+        </is>
+      </c>
+      <c r="C84" s="34" t="inlineStr">
+        <is>
+          <t>Ceramic Fibre Rope 10mm Dia x 30m
+(Temp 150-200°C)</t>
+        </is>
+      </c>
+      <c r="D84" s="33" t="inlineStr">
+        <is>
+          <t>ROL</t>
+        </is>
+      </c>
+      <c r="E84" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="F84" s="35" t="n">
+        <v>15789</v>
+      </c>
+      <c r="G84" s="35" t="n">
+        <v>63156</v>
+      </c>
+      <c r="H84" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I84" s="35" t="n">
+        <v>63156</v>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="36" t="inlineStr">
         <is>
           <t>GRAND TOTAL (All POs)</t>
         </is>
       </c>
-      <c r="I44" s="21" t="n">
-        <v>115103.1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="22" t="inlineStr">
+      <c r="I86" s="37" t="n">
+        <v>2622116.1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="38" t="inlineStr">
         <is>
           <t>PO SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="23" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="39" t="inlineStr">
         <is>
           <t>PO#</t>
         </is>
       </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="B89" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G47" s="23" t="inlineStr">
+      <c r="G89" s="39" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="H47" s="23" t="inlineStr">
+      <c r="H89" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="24" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="40" t="inlineStr">
         <is>
           <t>PO# 1183</t>
         </is>
       </c>
-      <c r="B48" s="25" t="inlineStr">
+      <c r="B90" s="41" t="inlineStr">
         <is>
           <t>Washing PVT — First Aid Items</t>
         </is>
       </c>
-      <c r="G48" s="24" t="inlineStr">
+      <c r="G90" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H48" s="26" t="inlineStr">
+      <c r="H90" s="42" t="inlineStr">
         <is>
           <t>PKR 35,890</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="24" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="40" t="inlineStr">
         <is>
           <t>PO# 17412</t>
         </is>
       </c>
-      <c r="B49" s="25" t="inlineStr">
+      <c r="B91" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Kitchen/Crockery</t>
         </is>
       </c>
-      <c r="G49" s="24" t="inlineStr">
+      <c r="G91" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H49" s="26" t="inlineStr">
+      <c r="H91" s="42" t="inlineStr">
         <is>
           <t>PKR 8,099</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="24" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="40" t="inlineStr">
         <is>
           <t>PO# 17426</t>
         </is>
       </c>
-      <c r="B50" s="25" t="inlineStr">
+      <c r="B92" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Plastic Jar</t>
         </is>
       </c>
-      <c r="G50" s="24" t="inlineStr">
+      <c r="G92" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H50" s="26" t="inlineStr">
+      <c r="H92" s="42" t="inlineStr">
         <is>
           <t>PKR 2,646</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="24" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="40" t="inlineStr">
         <is>
           <t>PO# 17427</t>
         </is>
       </c>
-      <c r="B51" s="25" t="inlineStr">
+      <c r="B93" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — First Aid Items</t>
         </is>
       </c>
-      <c r="G51" s="24" t="inlineStr">
+      <c r="G93" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H51" s="26" t="inlineStr">
+      <c r="H93" s="42" t="inlineStr">
         <is>
           <t>PKR 38,254</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="24" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="40" t="inlineStr">
         <is>
           <t>PO# 17186</t>
         </is>
       </c>
-      <c r="B52" s="25" t="inlineStr">
+      <c r="B94" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Plumbing Items</t>
         </is>
       </c>
-      <c r="G52" s="24" t="inlineStr">
+      <c r="G94" s="40" t="inlineStr">
         <is>
           <t>29-Jun-2026</t>
         </is>
       </c>
-      <c r="H52" s="26" t="inlineStr">
+      <c r="H94" s="42" t="inlineStr">
         <is>
           <t>PKR 19,215</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="24" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="40" t="inlineStr">
         <is>
           <t>PO# 1163</t>
         </is>
       </c>
-      <c r="B53" s="25" t="inlineStr">
+      <c r="B95" s="41" t="inlineStr">
         <is>
           <t>Washing PVT — Steel Kafgeer</t>
         </is>
       </c>
-      <c r="G53" s="24" t="inlineStr">
+      <c r="G95" s="40" t="inlineStr">
         <is>
           <t>30-Jun-2026</t>
         </is>
       </c>
-      <c r="H53" s="26" t="inlineStr">
+      <c r="H95" s="42" t="inlineStr">
         <is>
           <t>PKR 11,000</t>
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="40" t="inlineStr">
+        <is>
+          <t>PO# 17257</t>
+        </is>
+      </c>
+      <c r="B96" s="41" t="inlineStr">
+        <is>
+          <t>Cut to Pack PVT — Janitorial/Cleaning</t>
+        </is>
+      </c>
+      <c r="G96" s="40" t="inlineStr">
+        <is>
+          <t>29-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H96" s="42" t="inlineStr">
+        <is>
+          <t>PKR 760,293</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="40" t="inlineStr">
+        <is>
+          <t>PO# 17308</t>
+        </is>
+      </c>
+      <c r="B97" s="41" t="inlineStr">
+        <is>
+          <t>Cut to Pack PVT — Grocery/Entertainment</t>
+        </is>
+      </c>
+      <c r="G97" s="40" t="inlineStr">
+        <is>
+          <t>30-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H97" s="42" t="inlineStr">
+        <is>
+          <t>PKR 1,662,090</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="40" t="inlineStr">
+        <is>
+          <t>PO# 1194</t>
+        </is>
+      </c>
+      <c r="B98" s="41" t="inlineStr">
+        <is>
+          <t>Washing PVT — Production Consumables</t>
+        </is>
+      </c>
+      <c r="G98" s="40" t="inlineStr">
+        <is>
+          <t>06-Jul-2026</t>
+        </is>
+      </c>
+      <c r="H98" s="42" t="inlineStr">
+        <is>
+          <t>PKR 21,474</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="40" t="inlineStr">
+        <is>
+          <t>PO# 406</t>
+        </is>
+      </c>
+      <c r="B99" s="41" t="inlineStr">
+        <is>
+          <t>Utilities PVT — Mechanical Items</t>
+        </is>
+      </c>
+      <c r="G99" s="40" t="inlineStr">
+        <is>
+          <t>03-Jul-2026</t>
+        </is>
+      </c>
+      <c r="H99" s="42" t="inlineStr">
+        <is>
+          <t>PKR 63,156</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="B52:F52"/>
+  <mergeCells count="34">
+    <mergeCell ref="H91:I91"/>
+    <mergeCell ref="B91:F91"/>
+    <mergeCell ref="B90:F90"/>
+    <mergeCell ref="H93:I93"/>
+    <mergeCell ref="B93:F93"/>
+    <mergeCell ref="B96:F96"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="H49:I49"/>
-    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="H98:I98"/>
+    <mergeCell ref="B98:F98"/>
+    <mergeCell ref="H94:I94"/>
+    <mergeCell ref="H89:I89"/>
     <mergeCell ref="A4:I4"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="A72:I72"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A81:I81"/>
+    <mergeCell ref="A86:H86"/>
     <mergeCell ref="A28:I28"/>
+    <mergeCell ref="H90:I90"/>
     <mergeCell ref="A40:I40"/>
-    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="H99:I99"/>
+    <mergeCell ref="B99:F99"/>
+    <mergeCell ref="A83:I83"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="H96:I96"/>
+    <mergeCell ref="B92:F92"/>
+    <mergeCell ref="H95:I95"/>
+    <mergeCell ref="B95:F95"/>
+    <mergeCell ref="B89:F89"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="A88:I88"/>
+    <mergeCell ref="B94:F94"/>
+    <mergeCell ref="H97:I97"/>
+    <mergeCell ref="H92:I92"/>
+    <mergeCell ref="B97:F97"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add PO 76 (Denim Unit) mechanical items to buying sheet
Added 17 carpenter/mechanical items from PO 76 (Denim Unit, 30-Jun-2026)
to the mechanical category. Updated subtitle to 11 POs and added PO 76
to the summary section.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JrgSPE8qZmAUatRmCqrXMY
</commit_message>
<xml_diff>
--- a/Kashif_Buying_Sheet.xlsx
+++ b/Kashif_Buying_Sheet.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -684,7 +684,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dates: 29-Jun to 06-Jul-2026 | 10 POs | Deliver To: Main Store, Plot #8 Sector 27, Karachi</t>
+          <t>Dates: 29-Jun to 06-Jul-2026 | 11 POs | Deliver To: Main Store, Plot #8 Sector 27, Karachi</t>
         </is>
       </c>
     </row>
@@ -3416,301 +3416,954 @@
         <v>63156</v>
       </c>
     </row>
-    <row r="86" ht="28" customHeight="1">
-      <c r="A86" s="36" t="inlineStr">
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="33" t="n">
+        <v>74</v>
+      </c>
+      <c r="B85" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C85" s="34" t="inlineStr">
+        <is>
+          <t>Bench Vise / Wood Working Vice Set</t>
+        </is>
+      </c>
+      <c r="D85" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E85" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" s="35" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G85" s="35" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H85" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I85" s="35" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="33" t="n">
+        <v>75</v>
+      </c>
+      <c r="B86" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C86" s="34" t="inlineStr">
+        <is>
+          <t>C-Clamp Set</t>
+        </is>
+      </c>
+      <c r="D86" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E86" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F86" s="35" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G86" s="35" t="n">
+        <v>6240</v>
+      </c>
+      <c r="H86" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I86" s="35" t="n">
+        <v>6240</v>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="33" t="n">
+        <v>76</v>
+      </c>
+      <c r="B87" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C87" s="34" t="inlineStr">
+        <is>
+          <t>Center Punch Set</t>
+        </is>
+      </c>
+      <c r="D87" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E87" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="35" t="n">
+        <v>300</v>
+      </c>
+      <c r="G87" s="35" t="n">
+        <v>600</v>
+      </c>
+      <c r="H87" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I87" s="35" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="33" t="n">
+        <v>77</v>
+      </c>
+      <c r="B88" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C88" s="34" t="inlineStr">
+        <is>
+          <t>File Set (Rasp &amp; File Set / Ruff File - 10mm)</t>
+        </is>
+      </c>
+      <c r="D88" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E88" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" s="35" t="n">
+        <v>530</v>
+      </c>
+      <c r="G88" s="35" t="n">
+        <v>530</v>
+      </c>
+      <c r="H88" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I88" s="35" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="33" t="n">
+        <v>78</v>
+      </c>
+      <c r="B89" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C89" s="34" t="inlineStr">
+        <is>
+          <t>Flat Chisel Set</t>
+        </is>
+      </c>
+      <c r="D89" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E89" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" s="35" t="n">
+        <v>1875</v>
+      </c>
+      <c r="G89" s="35" t="n">
+        <v>1875</v>
+      </c>
+      <c r="H89" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I89" s="35" t="n">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="33" t="n">
+        <v>79</v>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C90" s="34" t="inlineStr">
+        <is>
+          <t>Hammer 1KG</t>
+        </is>
+      </c>
+      <c r="D90" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E90" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F90" s="35" t="n">
+        <v>480</v>
+      </c>
+      <c r="G90" s="35" t="n">
+        <v>2880</v>
+      </c>
+      <c r="H90" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I90" s="35" t="n">
+        <v>2880</v>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="33" t="n">
+        <v>80</v>
+      </c>
+      <c r="B91" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C91" s="34" t="inlineStr">
+        <is>
+          <t>Hammer 5KG</t>
+        </is>
+      </c>
+      <c r="D91" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E91" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" s="35" t="n">
+        <v>1125</v>
+      </c>
+      <c r="G91" s="35" t="n">
+        <v>1125</v>
+      </c>
+      <c r="H91" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I91" s="35" t="n">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="33" t="n">
+        <v>81</v>
+      </c>
+      <c r="B92" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C92" s="34" t="inlineStr">
+        <is>
+          <t>Hand Level 2'</t>
+        </is>
+      </c>
+      <c r="D92" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E92" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="35" t="n">
+        <v>313</v>
+      </c>
+      <c r="G92" s="35" t="n">
+        <v>626</v>
+      </c>
+      <c r="H92" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I92" s="35" t="n">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="33" t="n">
+        <v>82</v>
+      </c>
+      <c r="B93" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C93" s="34" t="inlineStr">
+        <is>
+          <t>Hole Saw Set 20mm to 50mm</t>
+        </is>
+      </c>
+      <c r="D93" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E93" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" s="35" t="n">
+        <v>938</v>
+      </c>
+      <c r="G93" s="35" t="n">
+        <v>938</v>
+      </c>
+      <c r="H93" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I93" s="35" t="n">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="33" t="n">
+        <v>83</v>
+      </c>
+      <c r="B94" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C94" s="34" t="inlineStr">
+        <is>
+          <t>Iron Chisel Rod 1'</t>
+        </is>
+      </c>
+      <c r="D94" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E94" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F94" s="35" t="n">
+        <v>570</v>
+      </c>
+      <c r="G94" s="35" t="n">
+        <v>3420</v>
+      </c>
+      <c r="H94" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I94" s="35" t="n">
+        <v>3420</v>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="33" t="n">
+        <v>84</v>
+      </c>
+      <c r="B95" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C95" s="34" t="inlineStr">
+        <is>
+          <t>Iron Chisel Rod 1.5'</t>
+        </is>
+      </c>
+      <c r="D95" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E95" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F95" s="35" t="n">
+        <v>570</v>
+      </c>
+      <c r="G95" s="35" t="n">
+        <v>3420</v>
+      </c>
+      <c r="H95" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I95" s="35" t="n">
+        <v>3420</v>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="33" t="n">
+        <v>85</v>
+      </c>
+      <c r="B96" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C96" s="34" t="inlineStr">
+        <is>
+          <t>Measuring Tape / Inch Tape 16FT</t>
+        </is>
+      </c>
+      <c r="D96" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E96" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F96" s="35" t="n">
+        <v>230</v>
+      </c>
+      <c r="G96" s="35" t="n">
+        <v>1380</v>
+      </c>
+      <c r="H96" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I96" s="35" t="n">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="33" t="n">
+        <v>86</v>
+      </c>
+      <c r="B97" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C97" s="34" t="inlineStr">
+        <is>
+          <t>Nail Punch Set</t>
+        </is>
+      </c>
+      <c r="D97" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E97" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" s="35" t="n">
+        <v>875</v>
+      </c>
+      <c r="G97" s="35" t="n">
+        <v>1750</v>
+      </c>
+      <c r="H97" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I97" s="35" t="n">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="33" t="n">
+        <v>87</v>
+      </c>
+      <c r="B98" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C98" s="34" t="inlineStr">
+        <is>
+          <t>Screw Extractor Set 3mm-6mm Total Brand</t>
+        </is>
+      </c>
+      <c r="D98" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E98" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" s="35" t="n">
+        <v>813</v>
+      </c>
+      <c r="G98" s="35" t="n">
+        <v>813</v>
+      </c>
+      <c r="H98" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I98" s="35" t="n">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="33" t="n">
+        <v>88</v>
+      </c>
+      <c r="B99" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C99" s="34" t="inlineStr">
+        <is>
+          <t>Try Square 2 Ft x 6 Inch (Steel)</t>
+        </is>
+      </c>
+      <c r="D99" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E99" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" s="35" t="n">
+        <v>500</v>
+      </c>
+      <c r="G99" s="35" t="n">
+        <v>500</v>
+      </c>
+      <c r="H99" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I99" s="35" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="33" t="n">
+        <v>89</v>
+      </c>
+      <c r="B100" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C100" s="34" t="inlineStr">
+        <is>
+          <t>Try Square Steel Type</t>
+        </is>
+      </c>
+      <c r="D100" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E100" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" s="35" t="n">
+        <v>350</v>
+      </c>
+      <c r="G100" s="35" t="n">
+        <v>700</v>
+      </c>
+      <c r="H100" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I100" s="35" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="33" t="n">
+        <v>90</v>
+      </c>
+      <c r="B101" s="33" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C101" s="34" t="inlineStr">
+        <is>
+          <t>Yato Screw Wrench Set</t>
+        </is>
+      </c>
+      <c r="D101" s="33" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="E101" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" s="35" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G101" s="35" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H101" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I101" s="35" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="36" t="inlineStr">
         <is>
           <t>GRAND TOTAL (All POs)</t>
         </is>
       </c>
-      <c r="I86" s="37" t="n">
-        <v>2622116.1</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="38" t="inlineStr">
+      <c r="I103" s="37" t="n">
+        <v>2656913.1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="38" t="inlineStr">
         <is>
           <t>PO SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="39" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="39" t="inlineStr">
         <is>
           <t>PO#</t>
         </is>
       </c>
-      <c r="B89" s="39" t="inlineStr">
+      <c r="B106" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G89" s="39" t="inlineStr">
+      <c r="G106" s="39" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="H89" s="39" t="inlineStr">
+      <c r="H106" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="40" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="40" t="inlineStr">
         <is>
           <t>PO# 1183</t>
         </is>
       </c>
-      <c r="B90" s="41" t="inlineStr">
+      <c r="B107" s="41" t="inlineStr">
         <is>
           <t>Washing PVT — First Aid Items</t>
         </is>
       </c>
-      <c r="G90" s="40" t="inlineStr">
+      <c r="G107" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H90" s="42" t="inlineStr">
+      <c r="H107" s="42" t="inlineStr">
         <is>
           <t>PKR 35,890</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="40" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="40" t="inlineStr">
         <is>
           <t>PO# 17412</t>
         </is>
       </c>
-      <c r="B91" s="41" t="inlineStr">
+      <c r="B108" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Kitchen/Crockery</t>
         </is>
       </c>
-      <c r="G91" s="40" t="inlineStr">
+      <c r="G108" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H91" s="42" t="inlineStr">
+      <c r="H108" s="42" t="inlineStr">
         <is>
           <t>PKR 8,099</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="40" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="40" t="inlineStr">
         <is>
           <t>PO# 17426</t>
         </is>
       </c>
-      <c r="B92" s="41" t="inlineStr">
+      <c r="B109" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Plastic Jar</t>
         </is>
       </c>
-      <c r="G92" s="40" t="inlineStr">
+      <c r="G109" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H92" s="42" t="inlineStr">
+      <c r="H109" s="42" t="inlineStr">
         <is>
           <t>PKR 2,646</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="40" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="40" t="inlineStr">
         <is>
           <t>PO# 17427</t>
         </is>
       </c>
-      <c r="B93" s="41" t="inlineStr">
+      <c r="B110" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — First Aid Items</t>
         </is>
       </c>
-      <c r="G93" s="40" t="inlineStr">
+      <c r="G110" s="40" t="inlineStr">
         <is>
           <t>02-Jul-2026</t>
         </is>
       </c>
-      <c r="H93" s="42" t="inlineStr">
+      <c r="H110" s="42" t="inlineStr">
         <is>
           <t>PKR 38,254</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="40" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="40" t="inlineStr">
         <is>
           <t>PO# 17186</t>
         </is>
       </c>
-      <c r="B94" s="41" t="inlineStr">
+      <c r="B111" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Plumbing Items</t>
         </is>
       </c>
-      <c r="G94" s="40" t="inlineStr">
+      <c r="G111" s="40" t="inlineStr">
         <is>
           <t>29-Jun-2026</t>
         </is>
       </c>
-      <c r="H94" s="42" t="inlineStr">
+      <c r="H111" s="42" t="inlineStr">
         <is>
           <t>PKR 19,215</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="40" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="40" t="inlineStr">
         <is>
           <t>PO# 1163</t>
         </is>
       </c>
-      <c r="B95" s="41" t="inlineStr">
+      <c r="B112" s="41" t="inlineStr">
         <is>
           <t>Washing PVT — Steel Kafgeer</t>
         </is>
       </c>
-      <c r="G95" s="40" t="inlineStr">
+      <c r="G112" s="40" t="inlineStr">
         <is>
           <t>30-Jun-2026</t>
         </is>
       </c>
-      <c r="H95" s="42" t="inlineStr">
+      <c r="H112" s="42" t="inlineStr">
         <is>
           <t>PKR 11,000</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="40" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="40" t="inlineStr">
         <is>
           <t>PO# 17257</t>
         </is>
       </c>
-      <c r="B96" s="41" t="inlineStr">
+      <c r="B113" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Janitorial/Cleaning</t>
         </is>
       </c>
-      <c r="G96" s="40" t="inlineStr">
+      <c r="G113" s="40" t="inlineStr">
         <is>
           <t>29-Jun-2026</t>
         </is>
       </c>
-      <c r="H96" s="42" t="inlineStr">
+      <c r="H113" s="42" t="inlineStr">
         <is>
           <t>PKR 760,293</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="40" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="40" t="inlineStr">
         <is>
           <t>PO# 17308</t>
         </is>
       </c>
-      <c r="B97" s="41" t="inlineStr">
+      <c r="B114" s="41" t="inlineStr">
         <is>
           <t>Cut to Pack PVT — Grocery/Entertainment</t>
         </is>
       </c>
-      <c r="G97" s="40" t="inlineStr">
+      <c r="G114" s="40" t="inlineStr">
         <is>
           <t>30-Jun-2026</t>
         </is>
       </c>
-      <c r="H97" s="42" t="inlineStr">
+      <c r="H114" s="42" t="inlineStr">
         <is>
           <t>PKR 1,662,090</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="40" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="40" t="inlineStr">
         <is>
           <t>PO# 1194</t>
         </is>
       </c>
-      <c r="B98" s="41" t="inlineStr">
+      <c r="B115" s="41" t="inlineStr">
         <is>
           <t>Washing PVT — Production Consumables</t>
         </is>
       </c>
-      <c r="G98" s="40" t="inlineStr">
+      <c r="G115" s="40" t="inlineStr">
         <is>
           <t>06-Jul-2026</t>
         </is>
       </c>
-      <c r="H98" s="42" t="inlineStr">
+      <c r="H115" s="42" t="inlineStr">
         <is>
           <t>PKR 21,474</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="40" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="40" t="inlineStr">
         <is>
           <t>PO# 406</t>
         </is>
       </c>
-      <c r="B99" s="41" t="inlineStr">
+      <c r="B116" s="41" t="inlineStr">
         <is>
           <t>Utilities PVT — Mechanical Items</t>
         </is>
       </c>
-      <c r="G99" s="40" t="inlineStr">
+      <c r="G116" s="40" t="inlineStr">
         <is>
           <t>03-Jul-2026</t>
         </is>
       </c>
-      <c r="H99" s="42" t="inlineStr">
+      <c r="H116" s="42" t="inlineStr">
         <is>
           <t>PKR 63,156</t>
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="40" t="inlineStr">
+        <is>
+          <t>PO# 76</t>
+        </is>
+      </c>
+      <c r="B117" s="41" t="inlineStr">
+        <is>
+          <t>Denim Unit — Mechanical / Carpenter Items</t>
+        </is>
+      </c>
+      <c r="G117" s="40" t="inlineStr">
+        <is>
+          <t>30-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H117" s="42" t="inlineStr">
+        <is>
+          <t>PKR 34,797</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="H91:I91"/>
-    <mergeCell ref="B91:F91"/>
-    <mergeCell ref="B90:F90"/>
-    <mergeCell ref="H93:I93"/>
-    <mergeCell ref="B93:F93"/>
-    <mergeCell ref="B96:F96"/>
+  <mergeCells count="36">
+    <mergeCell ref="B106:F106"/>
+    <mergeCell ref="B113:F113"/>
+    <mergeCell ref="B109:F109"/>
+    <mergeCell ref="H112:I112"/>
+    <mergeCell ref="B115:F115"/>
+    <mergeCell ref="A105:I105"/>
+    <mergeCell ref="A103:H103"/>
+    <mergeCell ref="H113:I113"/>
+    <mergeCell ref="H114:I114"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="H98:I98"/>
-    <mergeCell ref="B98:F98"/>
-    <mergeCell ref="H94:I94"/>
-    <mergeCell ref="H89:I89"/>
+    <mergeCell ref="H117:I117"/>
+    <mergeCell ref="B117:F117"/>
+    <mergeCell ref="B111:F111"/>
+    <mergeCell ref="B107:F107"/>
     <mergeCell ref="A4:I4"/>
+    <mergeCell ref="H108:I108"/>
+    <mergeCell ref="H110:I110"/>
     <mergeCell ref="A72:I72"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="A81:I81"/>
-    <mergeCell ref="A86:H86"/>
+    <mergeCell ref="H109:I109"/>
+    <mergeCell ref="H115:I115"/>
     <mergeCell ref="A28:I28"/>
-    <mergeCell ref="H90:I90"/>
+    <mergeCell ref="B116:F116"/>
+    <mergeCell ref="B112:F112"/>
     <mergeCell ref="A40:I40"/>
-    <mergeCell ref="H99:I99"/>
-    <mergeCell ref="B99:F99"/>
+    <mergeCell ref="B108:F108"/>
     <mergeCell ref="A83:I83"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="H96:I96"/>
-    <mergeCell ref="B92:F92"/>
-    <mergeCell ref="H95:I95"/>
-    <mergeCell ref="B95:F95"/>
-    <mergeCell ref="B89:F89"/>
+    <mergeCell ref="H111:I111"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A88:I88"/>
-    <mergeCell ref="B94:F94"/>
-    <mergeCell ref="H97:I97"/>
-    <mergeCell ref="H92:I92"/>
-    <mergeCell ref="B97:F97"/>
+    <mergeCell ref="B114:F114"/>
+    <mergeCell ref="H116:I116"/>
+    <mergeCell ref="H107:I107"/>
+    <mergeCell ref="B110:F110"/>
+    <mergeCell ref="H106:I106"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>